<commit_message>
Additonal scripts and results
</commit_message>
<xml_diff>
--- a/Extended PFAS PBK model/PC Literature.xlsx
+++ b/Extended PFAS PBK model/PC Literature.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fotis\Documents\GitHub\PFAS_PBK_models\Extended PFAS PBK model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10B733B8-4E69-40FB-862A-4D8841D10E01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9782145C-2DA1-4441-BB6B-1CC179D184A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{8CE04722-CFA5-4576-A31E-E29BF9086A2C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{8CE04722-CFA5-4576-A31E-E29BF9086A2C}"/>
   </bookViews>
   <sheets>
     <sheet name="Tissue to Blood" sheetId="1" r:id="rId1"/>
@@ -1107,9 +1107,9 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7" hidden="1" customWidth="1"/>
-    <col min="4" max="5" width="0" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="0" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="7" customWidth="1"/>
+    <col min="4" max="5" width="8.88671875" customWidth="1"/>
+    <col min="7" max="7" width="8.88671875" customWidth="1"/>
     <col min="8" max="8" width="20.44140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="22.88671875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="19.88671875" bestFit="1" customWidth="1"/>
@@ -1425,15 +1425,13 @@
   <dimension ref="A1:AT20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="0" hidden="1" customWidth="1"/>
+    <col min="2" max="4" width="8.88671875" customWidth="1"/>
     <col min="5" max="5" width="12.33203125" customWidth="1"/>
-    <col min="6" max="8" width="8.88671875" customWidth="1"/>
-    <col min="10" max="16" width="0" hidden="1" customWidth="1"/>
-    <col min="18" max="19" width="0" hidden="1" customWidth="1"/>
-    <col min="20" max="20" width="19.109375" bestFit="1" customWidth="1"/>
-    <col min="21" max="24" width="0" hidden="1" customWidth="1"/>
-    <col min="26" max="28" width="0" hidden="1" customWidth="1"/>
-    <col min="30" max="46" width="0" hidden="1" customWidth="1"/>
+    <col min="6" max="19" width="8.88671875" customWidth="1"/>
+    <col min="20" max="20" width="19.109375" customWidth="1"/>
+    <col min="21" max="27" width="8.88671875" customWidth="1"/>
+    <col min="28" max="28" width="12" bestFit="1" customWidth="1"/>
+    <col min="29" max="46" width="8.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:46" x14ac:dyDescent="0.3">

</xml_diff>